<commit_message>
submit: report the options a dropdown offered when nothing matched
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/job-tracker.xlsx
+++ b/tracking/job-tracker.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S42"/>
+  <dimension ref="A1:S47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="7" min="1" max="1"/>
@@ -2399,14 +2399,24 @@
           <t>AUD 185,000 base plus superannuation</t>
         </is>
       </c>
+      <c r="I28" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="J28" s="15" t="inlineStr">
         <is>
-          <t>To Apply</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="K28" s="15" t="inlineStr">
         <is>
-          <t>Approve + submit</t>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L28" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O28" s="15" t="inlineStr">
@@ -2461,14 +2471,24 @@
           <t>EUR 85,000 gross per year plus 8% holiday allowance</t>
         </is>
       </c>
+      <c r="I29" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="J29" s="15" t="inlineStr">
         <is>
-          <t>To Apply</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="K29" s="15" t="inlineStr">
         <is>
-          <t>Approve + submit</t>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L29" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O29" s="15" t="inlineStr">
@@ -2523,14 +2543,24 @@
           <t>AUD 185,000 base plus superannuation</t>
         </is>
       </c>
+      <c r="I30" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="J30" s="15" t="inlineStr">
         <is>
-          <t>To Apply</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="K30" s="15" t="inlineStr">
         <is>
-          <t>Approve + submit</t>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L30" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O30" s="15" t="inlineStr">
@@ -2957,19 +2987,39 @@
           <t>https://job-boards.greenhouse.io/adyen/jobs/7908806</t>
         </is>
       </c>
+      <c r="H37" s="15" t="inlineStr">
+        <is>
+          <t>EUR 85,000 gross per year plus 8% holiday allowance</t>
+        </is>
+      </c>
+      <c r="I37" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="J37" s="15" t="inlineStr">
         <is>
-          <t>To Apply</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="K37" s="15" t="inlineStr">
         <is>
-          <t>Tailor + fill</t>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L37" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O37" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
         </is>
       </c>
       <c r="P37" s="15" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="Q37" s="15" t="inlineStr">
@@ -3260,6 +3310,361 @@
       <c r="Q42" s="15" t="inlineStr">
         <is>
           <t>pipeline score 78.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>Deepjudge</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>Zurich HQ</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/deepjudge/2b8806be-d6d7-4929-9b0f-b2c09e197669/application</t>
+        </is>
+      </c>
+      <c r="H43" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base</t>
+        </is>
+      </c>
+      <c r="I43" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J43" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K43" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L43" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O43" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P43" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>Deepjudge</t>
+        </is>
+      </c>
+      <c r="B44" s="15" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="inlineStr">
+        <is>
+          <t>Zurich HQ</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G44" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/deepjudge/cbec610a-9fb7-4d86-bd3d-f97089a2d6c3/application</t>
+        </is>
+      </c>
+      <c r="H44" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base</t>
+        </is>
+      </c>
+      <c r="I44" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J44" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K44" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L44" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O44" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P44" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>Flow Traders</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G45" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/flowtraders/jobs/8090609</t>
+        </is>
+      </c>
+      <c r="H45" s="15" t="inlineStr">
+        <is>
+          <t>EUR 85,000 gross per year plus 8% holiday allowance</t>
+        </is>
+      </c>
+      <c r="I45" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J45" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K45" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L45" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O45" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P45" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>Hugging Face</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>Open-Source Machine Learning Engineer - EMEA Remote</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>Paris, France Remote</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>https://apply.workable.com/j/81B46579FE</t>
+        </is>
+      </c>
+      <c r="I46" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J46" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K46" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L46" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O46" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P46" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>Taktile</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>Senior Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>Berlin Office</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F47" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G47" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/taktile/d56d9c0d-5585-43d1-bc94-304bcc4ba11f/application</t>
+        </is>
+      </c>
+      <c r="H47" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base</t>
+        </is>
+      </c>
+      <c r="I47" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J47" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K47" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L47" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O47" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P47" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Self-healing submit: failed attempts turn missing required fields into review-page questions (no LLM), verification-code timeouts stay approved, 3rd failure lands in a 'Failed — needs a look' section with reason/screenshot/Retry; review run files approved items itself; one Telegram line per outcome
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/job-tracker.xlsx
+++ b/tracking/job-tracker.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S47"/>
+  <dimension ref="A1:S48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="7" min="1" max="1"/>
@@ -2615,14 +2615,24 @@
           <t>USD 200,000 base</t>
         </is>
       </c>
+      <c r="I31" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="J31" s="15" t="inlineStr">
         <is>
-          <t>To Apply</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="K31" s="15" t="inlineStr">
         <is>
-          <t>Approve + submit</t>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L31" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O31" s="15" t="inlineStr">
@@ -3663,6 +3673,78 @@
         </is>
       </c>
       <c r="P47" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>Research Engineer, Production Model Post-Training</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>Zürich, CH</t>
+        </is>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E48" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F48" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G48" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5112018008</t>
+        </is>
+      </c>
+      <c r="H48" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base</t>
+        </is>
+      </c>
+      <c r="I48" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J48" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K48" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L48" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O48" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P48" s="15" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>

</xml_diff>

<commit_message>
Workday: strip 'current step N of M' prefix (Review was not recognised and the Review button — Submit — was pressed on the submit leg), recognise 'already applied', page chrome never tagged, nameless re-find refused, consent wording in the acknowledgement rule
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/job-tracker.xlsx
+++ b/tracking/job-tracker.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S48"/>
+  <dimension ref="A1:S49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="7" min="1" max="1"/>
@@ -3750,6 +3750,78 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist, AI Engineering</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>Dublin, Ireland</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F49" s="15" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="G49" s="15" t="inlineStr">
+        <is>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Dublin-Ireland/Senior-AI-Engineer---Foundation-Models-and-Transformers-1_R-286224</t>
+        </is>
+      </c>
+      <c r="H49" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="I49" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J49" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K49" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L49" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O49" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P49" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q24"/>
   <hyperlinks>

</xml_diff>

<commit_message>
Applications, answers and trackers: new application folders, one stored answer
- answers.yaml: screening.confirm_form_statements (a form's "I confirm the
  statement above" box, answered from the profile instead of asked each time)
- learned.yaml: answers given on the phone since the last commit
- fifteen application folders (JD, notes, tailored resume sources)
- job and referral trackers as the pipeline left them

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/job-tracker.xlsx
+++ b/tracking/job-tracker.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S49"/>
+  <dimension ref="A1:S65"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="7" min="1" max="1"/>
@@ -3822,6 +3822,1063 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>Research Engineer</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E50" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F50" s="15" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="G50" s="15" t="inlineStr">
+        <is>
+          <t>https://adobe.wd5.myworkdayjobs.com/external_experienced/job/Seattle/Research-Engineer_R166886</t>
+        </is>
+      </c>
+      <c r="H50" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J50" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K50" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O50" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P50" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>Sr. Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E51" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F51" s="15" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="G51" s="15" t="inlineStr">
+        <is>
+          <t>https://adobe.wd5.myworkdayjobs.com/external_experienced/job/San-Francisco/Sr-Applied-AI-Engineer_R171752</t>
+        </is>
+      </c>
+      <c r="H51" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J51" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K51" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O51" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P51" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="15" t="inlineStr">
+        <is>
+          <t>Berkadia</t>
+        </is>
+      </c>
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>Senior Engineer - Machine Learning</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D52" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E52" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F52" s="15" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="G52" s="15" t="inlineStr">
+        <is>
+          <t>https://berkadia.wd1.myworkdayjobs.com/Berkadia/job/New-York-NY/Senior-Engineer---Machine-Learning_R-00021</t>
+        </is>
+      </c>
+      <c r="H52" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="I52" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J52" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K52" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L52" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O52" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P52" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="15" t="inlineStr">
+        <is>
+          <t>Capital One Careers</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="inlineStr">
+        <is>
+          <t>AI Engineer 4 (Gen AI Platform Services: Agentic AI, Agent Guardrails, Agent Evaluation, Agent Memory) at Capital One</t>
+        </is>
+      </c>
+      <c r="C53" s="15" t="inlineStr">
+        <is>
+          <t>- **Platform / How applying:** workday — ATS-critical, use the .docx</t>
+        </is>
+      </c>
+      <c r="D53" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E53" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F53" s="15" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="G53" s="15" t="inlineStr">
+        <is>
+          <t>https://capitalone.wd12.myworkdayjobs.com/Capital_One/job/San-Francisco--CA/AI-Engineer-4--Gen-AI-Platform-Services--Agentic-AI--Agent-Guardrails--Agent-Evaluation--Agent-Memory-_R1001053-1/apply</t>
+        </is>
+      </c>
+      <c r="H53" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base</t>
+        </is>
+      </c>
+      <c r="I53" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J53" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K53" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L53" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O53" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P53" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="15" t="inlineStr">
+        <is>
+          <t>Catawiki</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist - Machine Learning</t>
+        </is>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D54" s="15" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E54" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F54" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G54" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/catawiki/jobs/4994046</t>
+        </is>
+      </c>
+      <c r="H54" s="15" t="inlineStr">
+        <is>
+          <t>EUR 85,000 gross per year plus 8% holiday allowance</t>
+        </is>
+      </c>
+      <c r="J54" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K54" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O54" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P54" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="15" t="inlineStr">
+        <is>
+          <t>Takeaway</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>Senior Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>Amsterdam Office</t>
+        </is>
+      </c>
+      <c r="D55" s="15" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E55" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F55" s="15" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="G55" s="15" t="inlineStr">
+        <is>
+          <t>https://wd3.myworkdaysite.com/recruiting/takeaway/JET-ECS-R/job/Amsterdam-Office/Senior-Legal-Operation-Engineer_R_053008</t>
+        </is>
+      </c>
+      <c r="H55" s="15" t="inlineStr">
+        <is>
+          <t>EUR 85,000 gross per year plus 8% holiday allowance</t>
+        </is>
+      </c>
+      <c r="I55" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J55" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K55" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L55" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O55" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P55" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t>KONUX</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist (m/f/x)</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="D56" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E56" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F56" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G56" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/konux/jobs/7805858003</t>
+        </is>
+      </c>
+      <c r="H56" s="15" t="inlineStr">
+        <is>
+          <t>EUR 88,000 gross per year</t>
+        </is>
+      </c>
+      <c r="I56" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J56" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K56" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L56" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O56" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P56" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>Mercura</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="inlineStr">
+        <is>
+          <t>(Senior) AI/LLM Engineer</t>
+        </is>
+      </c>
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="D57" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E57" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F57" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G57" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/mercura/90bb4d91-9311-4d6c-a30b-a2d6dc783a13/application</t>
+        </is>
+      </c>
+      <c r="H57" s="15" t="inlineStr">
+        <is>
+          <t>EUR 88,000 gross per year</t>
+        </is>
+      </c>
+      <c r="I57" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J57" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K57" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L57" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O57" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P57" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="B58" s="15" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist</t>
+        </is>
+      </c>
+      <c r="C58" s="15" t="inlineStr">
+        <is>
+          <t>Cork, Ireland; Dublin, Ireland</t>
+        </is>
+      </c>
+      <c r="D58" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E58" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F58" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G58" s="15" t="inlineStr">
+        <is>
+          <t>https://www.mongodb.com/careers/job/?gh_jid=8135458</t>
+        </is>
+      </c>
+      <c r="H58" s="15" t="inlineStr">
+        <is>
+          <t>EUR 90,000 gross per year</t>
+        </is>
+      </c>
+      <c r="I58" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J58" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K58" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L58" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O58" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P58" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>Nvidia</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>Senior Research Scientist for Generative AI</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>US, CA, Santa Clara</t>
+        </is>
+      </c>
+      <c r="D59" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E59" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F59" s="15" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="G59" s="15" t="inlineStr">
+        <is>
+          <t>https://nvidia.wd5.myworkdayjobs.com/NVIDIAExternalCareerSite/job/US-CA-Santa-Clara/Senior-Research-Scientist-for-Generative-AI_JR2008124</t>
+        </is>
+      </c>
+      <c r="H59" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="I59" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J59" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K59" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L59" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O59" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P59" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="15" t="inlineStr">
+        <is>
+          <t>Openai</t>
+        </is>
+      </c>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>Applied AI Engineer, Startups (Codex)</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>Munich, Germany</t>
+        </is>
+      </c>
+      <c r="D60" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E60" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F60" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G60" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/e522c734-6e4e-4d69-80c1-d09d5144eab4/application</t>
+        </is>
+      </c>
+      <c r="H60" s="15" t="inlineStr">
+        <is>
+          <t>EUR 88,000 gross per year</t>
+        </is>
+      </c>
+      <c r="J60" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K60" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O60" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P60" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="15" t="inlineStr">
+        <is>
+          <t>Reflectionai</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
+          <t>Member of Technical Staff - Pre-Training</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D61" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E61" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F61" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G61" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/reflectionai/2c2b06f0-7897-4d22-9669-ec39e706d17a/application</t>
+        </is>
+      </c>
+      <c r="H61" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="I61" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="J61" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K61" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L61" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O61" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P61" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="15" t="inlineStr">
+        <is>
+          <t>Workday</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer - Payroll</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>USA, CA, Pleasanton</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E62" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F62" s="15" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="G62" s="15" t="inlineStr">
+        <is>
+          <t>https://workday.wd5.myworkdayjobs.com/Workday/job/USA-CA-Pleasanton/Machine-Learning-Engineer---Payroll_JR-0108977</t>
+        </is>
+      </c>
+      <c r="H62" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J62" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K62" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O62" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P62" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="15" t="inlineStr">
+        <is>
+          <t>Openai</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
+        <is>
+          <t>Applied AI Engineer, Codex</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>Munich, Germany</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E63" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F63" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G63" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/6a7cedbd-0a7c-4f3e-8389-55357ad444b3</t>
+        </is>
+      </c>
+      <c r="J63" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K63" s="15" t="inlineStr">
+        <is>
+          <t>Tailor + fill</t>
+        </is>
+      </c>
+      <c r="P63" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="Q63" s="15" t="inlineStr">
+        <is>
+          <t>pipeline score 87.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr">
+        <is>
+          <t>Workday</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>Ireland, Dublin</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E64" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F64" s="15" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="G64" s="15" t="inlineStr">
+        <is>
+          <t>https://workday.wd5.myworkdayjobs.com/Workday/job/Ireland-Dublin/Senior-AI-Engineer_JR-0108715</t>
+        </is>
+      </c>
+      <c r="J64" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K64" s="15" t="inlineStr">
+        <is>
+          <t>Tailor + fill</t>
+        </is>
+      </c>
+      <c r="P64" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="Q64" s="15" t="inlineStr">
+        <is>
+          <t>pipeline score 81.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="15" t="inlineStr">
+        <is>
+          <t>Helloprint</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer</t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+        </is>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E65" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F65" s="15" t="inlineStr">
+        <is>
+          <t>recruitee</t>
+        </is>
+      </c>
+      <c r="G65" s="15" t="inlineStr">
+        <is>
+          <t>https://helloprint.recruitee.com/o/senior-ai-engineer</t>
+        </is>
+      </c>
+      <c r="J65" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K65" s="15" t="inlineStr">
+        <is>
+          <t>Tailor + fill</t>
+        </is>
+      </c>
+      <c r="P65" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="Q65" s="15" t="inlineStr">
+        <is>
+          <t>pipeline score 81.2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q24"/>
   <hyperlinks>

</xml_diff>

<commit_message>
Filing fixes from the first full pipeline run
- after Submit: an emailed code is watched for on every poll (none → code-needed, not sent);
  a greyed-out Submit counts as still there; no sign-in while the outcome is watched
- account gate: no second try in a session after a refused sign-in
- type-ahead boxes: suggestions drawn as plain elements in the field are read and the
  value's entry picked (typing and search); a value the box drops when left is reported
- redo: a control is missing only if still missing once the page is redone; a call that
  found nothing is not recorded again; Add redone only for the numbered blocks missing;
  a section-less press is never skipped as a done Delete
- tailoring: one posting picked once per batch (two titles, one URL); explore cap in config
  (pipeline.explore_timeout_s, 2400s)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/job-tracker.xlsx
+++ b/tracking/job-tracker.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S65"/>
+  <dimension ref="A1:S81"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="7" min="1" max="1"/>
@@ -4131,14 +4131,24 @@
           <t>EUR 85,000 gross per year plus 8% holiday allowance</t>
         </is>
       </c>
+      <c r="I54" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="J54" s="15" t="inlineStr">
         <is>
-          <t>To Apply</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="K54" s="15" t="inlineStr">
         <is>
-          <t>Approve + submit</t>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L54" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O54" s="15" t="inlineStr">
@@ -4553,14 +4563,24 @@
           <t>EUR 88,000 gross per year</t>
         </is>
       </c>
+      <c r="I60" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="J60" s="15" t="inlineStr">
         <is>
-          <t>To Apply</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="K60" s="15" t="inlineStr">
         <is>
-          <t>Approve + submit</t>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L60" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O60" s="15" t="inlineStr">
@@ -4876,6 +4896,1048 @@
       <c r="Q65" s="15" t="inlineStr">
         <is>
           <t>pipeline score 81.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="15" t="inlineStr">
+        <is>
+          <t>Afterquery</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>Research Engineer</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E66" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F66" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G66" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/afterquery/ae665a77-b88d-418e-941a-6c3da870f052/application</t>
+        </is>
+      </c>
+      <c r="H66" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J66" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K66" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O66" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P66" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="inlineStr">
+        <is>
+          <t>Research Engineer, Code RL (Reinforcement Learning)</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco, CA | New York City, NY</t>
+        </is>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E67" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F67" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G67" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5254364008</t>
+        </is>
+      </c>
+      <c r="H67" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J67" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K67" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O67" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P67" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>Research Engineer, Life Sciences</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E68" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F68" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G68" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5265365008</t>
+        </is>
+      </c>
+      <c r="H68" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J68" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K68" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O68" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P68" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
+          <t>Research Engineer, Machine Learning (Reinforcement Learning)</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco, CA | New York City, NY</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E69" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F69" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G69" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4613568008</t>
+        </is>
+      </c>
+      <c r="H69" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J69" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K69" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O69" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P69" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>Research Engineer, Post-Training Model Evaluations</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco, CA | Seattle, WA</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E70" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F70" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G70" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5198255008</t>
+        </is>
+      </c>
+      <c r="H70" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J70" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K70" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O70" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P70" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>Research Engineer, RL Engineering</t>
+        </is>
+      </c>
+      <c r="C71" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco, CA | New York City, NY | Seattle, WA</t>
+        </is>
+      </c>
+      <c r="D71" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E71" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F71" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G71" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/4952051008</t>
+        </is>
+      </c>
+      <c r="H71" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="I71" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="J71" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K71" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L71" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="O71" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P71" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>Research Engineer, Takeoff Intel</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="inlineStr">
+        <is>
+          <t>Remote-Friendly (Travel Required) | San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E72" s="15" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F72" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G72" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5416882008</t>
+        </is>
+      </c>
+      <c r="H72" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J72" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K72" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O72" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P72" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>Exa</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer</t>
+        </is>
+      </c>
+      <c r="C73" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco, California</t>
+        </is>
+      </c>
+      <c r="D73" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E73" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F73" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G73" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/exa/8932d319-b456-4ee0-9efd-16d82be8de80/application</t>
+        </is>
+      </c>
+      <c r="H73" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J73" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K73" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O73" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P73" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="15" t="inlineStr">
+        <is>
+          <t>Figma</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>AI Applied Scientist</t>
+        </is>
+      </c>
+      <c r="C74" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco, CA • New York, NY • United States</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E74" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F74" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G74" s="15" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/figma/jobs/5707966004?gh_jid=5707966004</t>
+        </is>
+      </c>
+      <c r="H74" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="I74" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="J74" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K74" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L74" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="O74" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P74" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="15" t="inlineStr">
+        <is>
+          <t>Harvey</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="inlineStr">
+        <is>
+          <t>Research Engineer, Post-Training</t>
+        </is>
+      </c>
+      <c r="C75" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="D75" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E75" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F75" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G75" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/harvey/d78083d9-a203-4ae4-b4b9-454d65df3702/application</t>
+        </is>
+      </c>
+      <c r="H75" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="I75" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="J75" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K75" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L75" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="O75" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P75" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="15" t="inlineStr">
+        <is>
+          <t>Takeaway</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist</t>
+        </is>
+      </c>
+      <c r="C76" s="15" t="inlineStr">
+        <is>
+          <t>Amsterdam Office</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E76" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F76" s="15" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="G76" s="15" t="inlineStr">
+        <is>
+          <t>https://wd3.myworkdaysite.com/recruiting/takeaway/JET-ECS-R/job/Amsterdam-Office/Senior-Data-Scientist_R_053624</t>
+        </is>
+      </c>
+      <c r="H76" s="15" t="inlineStr">
+        <is>
+          <t>EUR 85,000 gross per year plus 8% holiday allowance</t>
+        </is>
+      </c>
+      <c r="J76" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K76" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O76" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P76" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="15" t="inlineStr">
+        <is>
+          <t>Lio</t>
+        </is>
+      </c>
+      <c r="B77" s="15" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer (all genders)</t>
+        </is>
+      </c>
+      <c r="C77" s="15" t="inlineStr">
+        <is>
+          <t>Munich Office</t>
+        </is>
+      </c>
+      <c r="D77" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E77" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F77" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G77" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/lio/8e037444-9a05-4470-b1a1-eeeee26c8815/application</t>
+        </is>
+      </c>
+      <c r="H77" s="15" t="inlineStr">
+        <is>
+          <t>EUR 88,000 gross per year</t>
+        </is>
+      </c>
+      <c r="I77" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J77" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K77" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L77" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="O77" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P77" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="15" t="inlineStr">
+        <is>
+          <t>Openai</t>
+        </is>
+      </c>
+      <c r="B78" s="15" t="inlineStr">
+        <is>
+          <t>Research Engineer, Codex</t>
+        </is>
+      </c>
+      <c r="C78" s="15" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="D78" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E78" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F78" s="15" t="inlineStr">
+        <is>
+          <t>ashby</t>
+        </is>
+      </c>
+      <c r="G78" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/793964ae-d40b-45e3-9798-84f4b6da48c5/application</t>
+        </is>
+      </c>
+      <c r="H78" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="I78" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="J78" s="15" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="K78" s="15" t="inlineStr">
+        <is>
+          <t>Follow up if no reply</t>
+        </is>
+      </c>
+      <c r="L78" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="O78" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P78" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="15" t="inlineStr">
+        <is>
+          <t>Sonarsource</t>
+        </is>
+      </c>
+      <c r="B79" s="15" t="inlineStr">
+        <is>
+          <t>AI Research Engineer</t>
+        </is>
+      </c>
+      <c r="C79" s="15" t="inlineStr">
+        <is>
+          <t>Geneva</t>
+        </is>
+      </c>
+      <c r="D79" s="15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E79" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F79" s="15" t="inlineStr">
+        <is>
+          <t>lever</t>
+        </is>
+      </c>
+      <c r="G79" s="15" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/sonarsource/a0535931-bce3-4159-b43d-15ca3eb4d17f</t>
+        </is>
+      </c>
+      <c r="H79" s="15" t="inlineStr">
+        <is>
+          <t>CHF 155,000 gross per year</t>
+        </is>
+      </c>
+      <c r="J79" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K79" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O79" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P79" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="15" t="inlineStr">
+        <is>
+          <t>Turing</t>
+        </is>
+      </c>
+      <c r="B80" s="15" t="inlineStr">
+        <is>
+          <t>Senior Research Engineer, SWE</t>
+        </is>
+      </c>
+      <c r="C80" s="15" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D80" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E80" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F80" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G80" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/turing/jobs/5703798004</t>
+        </is>
+      </c>
+      <c r="H80" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J80" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K80" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O80" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P80" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="15" t="inlineStr">
+        <is>
+          <t>Turing</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="inlineStr">
+        <is>
+          <t>Senior Research Engineer, Frontier Data</t>
+        </is>
+      </c>
+      <c r="C81" s="15" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E81" s="15" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F81" s="15" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
+      <c r="G81" s="15" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/turing/jobs/6198595004</t>
+        </is>
+      </c>
+      <c r="H81" s="15" t="inlineStr">
+        <is>
+          <t>USD 200,000 base (open on total comp / equity mix)</t>
+        </is>
+      </c>
+      <c r="J81" s="15" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="K81" s="15" t="inlineStr">
+        <is>
+          <t>Approve + submit</t>
+        </is>
+      </c>
+      <c r="O81" s="15" t="inlineStr">
+        <is>
+          <t>sunil_resume.docx</t>
+        </is>
+      </c>
+      <c r="P81" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>

</xml_diff>